<commit_message>
Carga de nuevos productos al catálogo
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\Pagina Web Tecnocodys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A81708FE-9AE6-4183-92EA-89434F4DA9FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C1AC0F-2DBE-4831-9178-1043B4F2C7FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{D6650EB6-C58A-4F11-A148-31C065CE3CEC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7161" uniqueCount="3645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14322" uniqueCount="3645">
   <si>
     <t>CODIGO</t>
   </si>
@@ -12063,7 +12063,7 @@
         <v>12910</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>